<commit_message>
Update machine serial input
</commit_message>
<xml_diff>
--- a/machine_ids.xlsx
+++ b/machine_ids.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vedantp_ithena\Desktop\AMF Solid Edge Clean Up Automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ronits_ithena\Documents\AMF 3D Solid Edge Automation\amf_cleanup_automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27724009-581A-4C43-B1E0-DC5F83F847A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,21 +19,36 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>SR_NO</t>
   </si>
   <si>
-    <t>20494-1000ME</t>
+    <t>23251-1000UF</t>
   </si>
   <si>
-    <t>21437-1011ME</t>
+    <t xml:space="preserve">23251-1000ME  </t>
+  </si>
+  <si>
+    <t>23251-1002UF</t>
+  </si>
+  <si>
+    <t>23251-1002ME</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 20578-1000 ME</t>
+  </si>
+  <si>
+    <t>20578-1001 ME</t>
+  </si>
+  <si>
+    <t>24253-1000ME</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -132,8 +146,8 @@
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="Normal 3" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Normal 3" xfId="2"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -345,7 +359,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -361,29 +375,39 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>2</v>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4"/>
-    </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4"/>
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4"/>
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4"/>
+      <c r="A8" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="4"/>

</xml_diff>